<commit_message>
[20240414] Ejercicios práctica 01
</commit_message>
<xml_diff>
--- a/05_EXAMENES/zip_examen_prueba_01/ejercicios_practicos_propuestos_v2.xlsx
+++ b/05_EXAMENES/zip_examen_prueba_01/ejercicios_practicos_propuestos_v2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jorgejuvenalcamposferreira/Documents/GitHub/TC2001B.601-Ciencia-de-datos-ene-jun-2026/05_EXAMENES/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jorgejuvenalcamposferreira/Documents/GitHub/TC2001B.601-Ciencia-de-datos-ene-jun-2026/05_EXAMENES/zip_examen_prueba_01/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B0685A-3B06-6941-B063-A05A549913DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B8D486D-8BA0-DC45-A5B8-8C69D34674CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="68800" windowHeight="26600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ejercicios v2" sheetId="1" r:id="rId1"/>
@@ -901,7 +901,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" ht="64" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
@@ -942,7 +942,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" ht="64" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>25</v>
       </c>
@@ -983,7 +983,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" ht="80" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>36</v>
       </c>
@@ -1024,7 +1024,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" ht="64" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>48</v>
       </c>
@@ -1065,7 +1065,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="80" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="64" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>59</v>
       </c>
@@ -1106,7 +1106,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="112" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="80" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>69</v>
       </c>
@@ -1147,7 +1147,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="80" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>80</v>
       </c>
@@ -1188,7 +1188,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" ht="80" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>89</v>
       </c>
@@ -1229,7 +1229,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="64" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>100</v>
       </c>
@@ -1270,7 +1270,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" ht="80" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>110</v>
       </c>
@@ -1311,7 +1311,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="112" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" ht="80" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>119</v>
       </c>
@@ -1352,7 +1352,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="96" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" ht="80" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>130</v>
       </c>

</xml_diff>